<commit_message>
Tecnicas dinamica - 3pc
</commit_message>
<xml_diff>
--- a/Sistema de transporte/data.xlsx
+++ b/Sistema de transporte/data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unipe-my.sharepoint.com/personal/pedro_castillo_s_uni_pe/Documents/Desktop/UNI/8vo ciclo/Taller de Dinamica de Sistemas/Taller-de-DS/Sistema de transporte/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\piter\OneDrive\Escritorio\UNI\8VO CICLO\TALLER DE DINAMICA DE SISTEMAS\Sistema de transporte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_AD4D2F04E46CFB4ACB3E20FF2D90CB3E683EDF15" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{756356CE-452B-4EF0-B933-B9BECCD74BE6}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEDF07DD-86F9-4018-ABB9-4D2208BF1A91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="345" yWindow="1470" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6348" yWindow="5448" windowWidth="8928" windowHeight="3324" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -388,9 +388,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N102"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -434,7 +434,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -478,7 +478,7 @@
         <v>0.08</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -522,7 +522,7 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -566,7 +566,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -610,7 +610,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
@@ -654,7 +654,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>5</v>
       </c>
@@ -698,7 +698,7 @@
         <v>0.17</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -742,7 +742,7 @@
         <v>0.19</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -786,7 +786,7 @@
         <v>0.21</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -830,7 +830,7 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
@@ -874,7 +874,7 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10</v>
       </c>
@@ -918,7 +918,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>11</v>
       </c>
@@ -962,7 +962,7 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>12</v>
       </c>
@@ -1006,7 +1006,7 @@
         <v>0.27</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>13</v>
       </c>
@@ -1050,7 +1050,7 @@
         <v>0.28000000000000003</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>14</v>
       </c>
@@ -1094,7 +1094,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>15</v>
       </c>
@@ -1138,7 +1138,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>16</v>
       </c>
@@ -1182,7 +1182,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>17</v>
       </c>
@@ -1226,7 +1226,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>18</v>
       </c>
@@ -1270,7 +1270,7 @@
         <v>0.31</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>19</v>
       </c>
@@ -1314,7 +1314,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>20</v>
       </c>
@@ -1358,7 +1358,7 @@
         <v>0.32</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>21</v>
       </c>
@@ -1402,7 +1402,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>22</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>23</v>
       </c>
@@ -1490,7 +1490,7 @@
         <v>0.33</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>24</v>
       </c>
@@ -1534,7 +1534,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>25</v>
       </c>
@@ -1578,7 +1578,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>26</v>
       </c>
@@ -1622,7 +1622,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>27</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>28</v>
       </c>
@@ -1710,7 +1710,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>29</v>
       </c>
@@ -1754,7 +1754,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>30</v>
       </c>
@@ -1798,7 +1798,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>31</v>
       </c>
@@ -1842,7 +1842,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>32</v>
       </c>
@@ -1886,7 +1886,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>33</v>
       </c>
@@ -1930,7 +1930,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>34</v>
       </c>
@@ -1974,7 +1974,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>35</v>
       </c>
@@ -2018,7 +2018,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>36</v>
       </c>
@@ -2062,7 +2062,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>37</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>38</v>
       </c>
@@ -2150,7 +2150,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>39</v>
       </c>
@@ -2194,7 +2194,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>40</v>
       </c>
@@ -2238,7 +2238,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>41</v>
       </c>
@@ -2282,7 +2282,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>42</v>
       </c>
@@ -2326,7 +2326,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>43</v>
       </c>
@@ -2370,7 +2370,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>44</v>
       </c>
@@ -2414,7 +2414,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>45</v>
       </c>
@@ -2458,7 +2458,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>46</v>
       </c>
@@ -2502,7 +2502,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>47</v>
       </c>
@@ -2546,7 +2546,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>48</v>
       </c>
@@ -2590,7 +2590,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>49</v>
       </c>
@@ -2634,7 +2634,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>50</v>
       </c>
@@ -2678,7 +2678,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>51</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>52</v>
       </c>
@@ -2766,7 +2766,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>53</v>
       </c>
@@ -2810,7 +2810,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>54</v>
       </c>
@@ -2854,7 +2854,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>55</v>
       </c>
@@ -2898,7 +2898,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>56</v>
       </c>
@@ -2942,7 +2942,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>57</v>
       </c>
@@ -2986,7 +2986,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>58</v>
       </c>
@@ -3030,7 +3030,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>59</v>
       </c>
@@ -3074,7 +3074,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>60</v>
       </c>
@@ -3118,7 +3118,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>61</v>
       </c>
@@ -3162,7 +3162,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>62</v>
       </c>
@@ -3206,7 +3206,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>63</v>
       </c>
@@ -3250,7 +3250,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>64</v>
       </c>
@@ -3294,7 +3294,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>65</v>
       </c>
@@ -3338,7 +3338,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>66</v>
       </c>
@@ -3382,7 +3382,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>67</v>
       </c>
@@ -3426,7 +3426,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>68</v>
       </c>
@@ -3470,7 +3470,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>69</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>70</v>
       </c>
@@ -3558,7 +3558,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>71</v>
       </c>
@@ -3602,7 +3602,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>72</v>
       </c>
@@ -3646,7 +3646,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>73</v>
       </c>
@@ -3690,7 +3690,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>74</v>
       </c>
@@ -3734,7 +3734,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>75</v>
       </c>
@@ -3778,7 +3778,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>76</v>
       </c>
@@ -3822,7 +3822,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>77</v>
       </c>
@@ -3866,7 +3866,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>78</v>
       </c>
@@ -3910,7 +3910,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>79</v>
       </c>
@@ -3954,7 +3954,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>80</v>
       </c>
@@ -3998,7 +3998,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>81</v>
       </c>
@@ -4042,7 +4042,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>82</v>
       </c>
@@ -4086,7 +4086,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>83</v>
       </c>
@@ -4130,7 +4130,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>84</v>
       </c>
@@ -4174,7 +4174,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>85</v>
       </c>
@@ -4218,7 +4218,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>86</v>
       </c>
@@ -4262,7 +4262,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>87</v>
       </c>
@@ -4306,7 +4306,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>88</v>
       </c>
@@ -4350,7 +4350,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>89</v>
       </c>
@@ -4394,7 +4394,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>90</v>
       </c>
@@ -4438,7 +4438,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>91</v>
       </c>
@@ -4482,7 +4482,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>92</v>
       </c>
@@ -4526,7 +4526,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>93</v>
       </c>
@@ -4570,7 +4570,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>94</v>
       </c>
@@ -4614,7 +4614,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>95</v>
       </c>
@@ -4658,7 +4658,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="98" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>96</v>
       </c>
@@ -4702,7 +4702,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>97</v>
       </c>
@@ -4746,7 +4746,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>98</v>
       </c>
@@ -4790,7 +4790,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>99</v>
       </c>
@@ -4834,7 +4834,7 @@
         <v>0.36</v>
       </c>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>14</v>
       </c>

</xml_diff>